<commit_message>
chore: update test plan and remove stale lock file
</commit_message>
<xml_diff>
--- a/test_plan.xlsx
+++ b/test_plan.xlsx
@@ -1399,6 +1399,11 @@
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A48:F48"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="E3 E4 E5 E6 E7 E8 E9 E10 E14 E15 E16 E17 E18 E19 E20 E21 E25 E26 E27 E28 E29 E30 E31 E35 E36 E37 E38 E42 E43 E44 E45 E49 E50 E51 E52 E53 E54 E55 E59 E60 E61 E62 E63 E64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list (Yes or No)" promptTitle="Passed? (Yes/No)" prompt="Please select Yes or No" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>